<commit_message>
adding the pmas evolution analysis
</commit_message>
<xml_diff>
--- a/ressources/labels_questions_others.xlsx
+++ b/ressources/labels_questions_others.xlsx
@@ -1,352 +1,359 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted-my.sharepoint.com/personal/giovanni_giuliari_impact-initiatives_org/Documents/04_job_quality_assurance/03.capacity_building/03.CAR support/07.JMMI_script/REACH_CAR_JMMI_scripts/rca_jmmi_dashboard/ressources/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_B9923127ED9925EDF80723FA5F3D011832187E19" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E62194B5-B4F0-4E99-BB5E-FE41D3798AA9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ref_question</t>
-  </si>
-  <si>
-    <t xml:space="preserve">full_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">organisation_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">organisation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nom de l'organisation partenaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">infrastructure_shop_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">infrastructure_shop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comment décrirez-vous votre infrastructure de commerce sur le marché ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">shop_category_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">shop_category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les catégories de produits vendus par ce commerçant?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">food_supplier_unique_reason_other_ctgy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">food_supplier_unique_reason_ctgy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourquoi dépendez-vous d'un seul fournisseur pour les articles alimentaires que vous vendez ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_food_restock_difficulties_border_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">food_restock_difficulties_reason_ctgy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si oui, Quelles sont les causes du retard dans l'acheminement ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_food_restock_difficulties_border_other_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nfi_supplier_unique_reason_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nfi_supplier_unique_reason</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourquoi dépendez-vous d'un seul fournisseur pour les articles non alimentaires que vous vendez ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nfi_restock_difficullties_border</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nfi_restock_difficulties_item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nfi_restock_difficulties_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wash_supplier_unique_reason_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Veuillez préciser :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wash_restock_difficullties_border</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wash_restock_difficulties_item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wash_restock_difficulties_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire_combustion_supplier_unique_reason_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire_combustion_supplier_unique_reason</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourquoi dépendez-vous d'un seul fournisseur pour les produits combustibles que vous vendez ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire_combustion_restock_difficullties_border</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire_combustion_restock_difficulties_item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire_combustion_restock_difficulties_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_costumer_number_reduction_reasons_other_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_costumer_number_reduction_reasons_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les causes de la réduction du nombre de vos clients ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_any_shop_closed_in_marketplace_other_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_any_shop_closed_in_marketplace_reasons_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les causes de la fermeture de leur commerce ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_transportation_cost_wharehouse_reason_other_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_transportation_cost_wharehouse_reason_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A quoi est due cette augmentation du prix pour transporter vos marchandises de votre entrepôt au marché ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_transportation_cost_change_reason_other_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_transportation_cost_change_reason_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A quoi est due cette augmentation du prix pour transporter vos marchandises de chez le fournisseur, jusqu'à votre entrepôt ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_ac3_physical_access_mkt_discrimination_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_ac3_physical_access_mkt_discrimination_so</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Au cours du dernier mois, y a-t-il eu des groupes de personnes qui ont parfois évité de venir sur ce marché en raison de la discrimination, de l'exclusion ou parce qu'ils ne se sentaient pas les bienvenus ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_ac4_physical_access_security_issues_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_ac4_physical_access_security_issues_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quels types d'incidents de sécurité ou de sûreté avez-vous observés ou entendus ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_ac1_physical_access_mkt_issues_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autres raisons d'accès physique (veuillez préciser)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_re4_shop_operational_difficulties_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_re4_shop_operational_difficulties_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Éprouvez-vous actuellement des difficultés à maintenir votre entreprise opérationnelle et approvisionnée ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_af2_financial_challenges_customers_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_af2_financial_challenges_customers_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les clients de votre entreprise font-ils face à des difficultés financières lorsqu’ils se rendent chez vous ou qu’ils paient les marchandises dont ils ont besoin ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_in2_available_storage_facility_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_in2_available_storage_facility_so</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Au cours des derniers 7 jours, avez-vous eu accès à une installation d’entreposage verrouillée et sécurisée dans votre établissement commercial ou votre marché ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_af3_price_forecasting_noability_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_af3_price_forecasting_noability_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les raisons principales expliquant pourquoi vous auriez des difficultés à donner une estimation précise des prix pratiqués par vos fournisseurs le mois prochain ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_in3_accepted_payment_modality_other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mfs_in3_accepted_payment_modality_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quels types de paiement avez-vous acceptés de la part de vos clients ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_risque_type_paiement_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_risque_type_paiement_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quel est le risque associé aux types de paiement que vous avez sélectionnés ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_type_paiement_refusee_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_type_paiement_refusee_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y a-t-il des types de paiement que vous n'avez pas pu ou pas voulu accepter de la part de vos clients ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_difficulte_type_paiement_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_difficulte_type_paiement_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourquoi ces types de paiement sont-ils difficiles à accepter pour vous ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_existence_service_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_existence_service_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y a-t-il des services de transfet monétaire (banques, micro finance, mobile money) dans votre commune, et si oui lesquelles ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_argent_mobile_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_argent_mobile_so</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comment décririez-vous votre niveau actuel d'accès à l'argent mobile ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_psf_informel_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_psf_informel_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Au cours des 30 derniers jours, quels services ou moyens avez-vous utilisés pour accéder à des espèces ou effectuer des transferts d'argent ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_especes_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_acces_especes_so</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comment décririez-vous votre niveau actuel d'accès aux espèces ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_equite_distribution_cva_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_equite_distribution_cva_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À votre avis, les habitants de cette commune estiment-ils que les transferts monétaires (CVA) sont distribués de manière juste et équitable ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_preference_coupon_cva_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_preference_coupon_cva_so</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si vous deviez travailler avec un fournisseur d'aide financière humanitaire (CVA), quel serait votre type de coupon préféré ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_risque_cva_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_risque_cva_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À votre avis, existe-t-il des risques associés aux transferts monétaires ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_tensions_sociales_cva_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_tensions_sociales_cva_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si « Tensions sociales », quelles sont les tensions sociales qui découlent des transferts monétaires ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_impact_cva_autre_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_impact_cva_sm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quel serait l'impact de la fourniture d'une aide monétaire humanitaire aux ménages de cette commune sur votre commerce et sur le marché local ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAR_cfa_info_supplementaire_tx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avez-vous des informations supplémentaires que vous souhaiteriez partager concernant le marché et votre perception de l'aide financière humanitaire (CVA) qui n'auraient pas été abordées dans cette enquête ?</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="109">
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>ref_question</t>
+  </si>
+  <si>
+    <t>full_label</t>
+  </si>
+  <si>
+    <t>organisation_other</t>
+  </si>
+  <si>
+    <t>organisation</t>
+  </si>
+  <si>
+    <t>Nom de l'organisation partenaire</t>
+  </si>
+  <si>
+    <t>infrastructure_shop_other</t>
+  </si>
+  <si>
+    <t>infrastructure_shop</t>
+  </si>
+  <si>
+    <t>Comment décrirez-vous votre infrastructure de commerce sur le marché ?</t>
+  </si>
+  <si>
+    <t>shop_category_other</t>
+  </si>
+  <si>
+    <t>shop_category</t>
+  </si>
+  <si>
+    <t>Quelles sont les catégories de produits vendus par ce commerçant?</t>
+  </si>
+  <si>
+    <t>food_supplier_unique_reason_other_ctgy</t>
+  </si>
+  <si>
+    <t>food_supplier_unique_reason_ctgy</t>
+  </si>
+  <si>
+    <t>Pourquoi dépendez-vous d'un seul fournisseur pour les articles alimentaires que vous vendez ?</t>
+  </si>
+  <si>
+    <t>CAR_food_restock_difficulties_border_tx</t>
+  </si>
+  <si>
+    <t>food_restock_difficulties_reason_ctgy</t>
+  </si>
+  <si>
+    <t>Si oui, Quelles sont les causes du retard dans l'acheminement ?</t>
+  </si>
+  <si>
+    <t>CAR_food_restock_difficulties_border_other_tx</t>
+  </si>
+  <si>
+    <t>nfi_supplier_unique_reason_other</t>
+  </si>
+  <si>
+    <t>nfi_supplier_unique_reason</t>
+  </si>
+  <si>
+    <t>Pourquoi dépendez-vous d'un seul fournisseur pour les articles non alimentaires que vous vendez ?</t>
+  </si>
+  <si>
+    <t>nfi_restock_difficullties_border</t>
+  </si>
+  <si>
+    <t>nfi_restock_difficulties_item</t>
+  </si>
+  <si>
+    <t>nfi_restock_difficulties_other</t>
+  </si>
+  <si>
+    <t>wash_supplier_unique_reason_other</t>
+  </si>
+  <si>
+    <t>Veuillez préciser :</t>
+  </si>
+  <si>
+    <t>wash_restock_difficullties_border</t>
+  </si>
+  <si>
+    <t>wash_restock_difficulties_item</t>
+  </si>
+  <si>
+    <t>wash_restock_difficulties_other</t>
+  </si>
+  <si>
+    <t>fire_combustion_supplier_unique_reason_other</t>
+  </si>
+  <si>
+    <t>fire_combustion_supplier_unique_reason</t>
+  </si>
+  <si>
+    <t>Pourquoi dépendez-vous d'un seul fournisseur pour les produits combustibles que vous vendez ?</t>
+  </si>
+  <si>
+    <t>fire_combustion_restock_difficullties_border</t>
+  </si>
+  <si>
+    <t>fire_combustion_restock_difficulties_item</t>
+  </si>
+  <si>
+    <t>fire_combustion_restock_difficulties_other</t>
+  </si>
+  <si>
+    <t>CAR_costumer_number_reduction_reasons_other_tx</t>
+  </si>
+  <si>
+    <t>CAR_costumer_number_reduction_reasons_sm</t>
+  </si>
+  <si>
+    <t>Quelles sont les causes de la réduction du nombre de vos clients ?</t>
+  </si>
+  <si>
+    <t>CAR_any_shop_closed_in_marketplace_other_tx</t>
+  </si>
+  <si>
+    <t>CAR_any_shop_closed_in_marketplace_reasons_sm</t>
+  </si>
+  <si>
+    <t>Quelles sont les causes de la fermeture de leur commerce ?</t>
+  </si>
+  <si>
+    <t>CAR_transportation_cost_wharehouse_reason_other_tx</t>
+  </si>
+  <si>
+    <t>CAR_transportation_cost_wharehouse_reason_sm</t>
+  </si>
+  <si>
+    <t>A quoi est due cette augmentation du prix pour transporter vos marchandises de votre entrepôt au marché ?</t>
+  </si>
+  <si>
+    <t>CAR_transportation_cost_change_reason_other_tx</t>
+  </si>
+  <si>
+    <t>CAR_transportation_cost_change_reason_sm</t>
+  </si>
+  <si>
+    <t>A quoi est due cette augmentation du prix pour transporter vos marchandises de chez le fournisseur, jusqu'à votre entrepôt ?</t>
+  </si>
+  <si>
+    <t>mfs_ac3_physical_access_mkt_discrimination_other</t>
+  </si>
+  <si>
+    <t>mfs_ac3_physical_access_mkt_discrimination_so</t>
+  </si>
+  <si>
+    <t>Au cours du dernier mois, y a-t-il eu des groupes de personnes qui ont parfois évité de venir sur ce marché en raison de la discrimination, de l'exclusion ou parce qu'ils ne se sentaient pas les bienvenus ?</t>
+  </si>
+  <si>
+    <t>mfs_ac4_physical_access_security_issues_other</t>
+  </si>
+  <si>
+    <t>mfs_ac4_physical_access_security_issues_sm</t>
+  </si>
+  <si>
+    <t>Quels types d'incidents de sécurité ou de sûreté avez-vous observés ou entendus ?</t>
+  </si>
+  <si>
+    <t>mfs_ac1_physical_access_mkt_issues_other</t>
+  </si>
+  <si>
+    <t>Autres raisons d'accès physique (veuillez préciser)</t>
+  </si>
+  <si>
+    <t>mfs_re4_shop_operational_difficulties_other</t>
+  </si>
+  <si>
+    <t>mfs_re4_shop_operational_difficulties_sm</t>
+  </si>
+  <si>
+    <t>Éprouvez-vous actuellement des difficultés à maintenir votre entreprise opérationnelle et approvisionnée ?</t>
+  </si>
+  <si>
+    <t>mfs_af2_financial_challenges_customers_other</t>
+  </si>
+  <si>
+    <t>mfs_af2_financial_challenges_customers_sm</t>
+  </si>
+  <si>
+    <t>Les clients de votre entreprise font-ils face à des difficultés financières lorsqu’ils se rendent chez vous ou qu’ils paient les marchandises dont ils ont besoin ?</t>
+  </si>
+  <si>
+    <t>mfs_in2_available_storage_facility_other</t>
+  </si>
+  <si>
+    <t>mfs_in2_available_storage_facility_so</t>
+  </si>
+  <si>
+    <t>Au cours des derniers 7 jours, avez-vous eu accès à une installation d’entreposage verrouillée et sécurisée dans votre établissement commercial ou votre marché ?</t>
+  </si>
+  <si>
+    <t>mfs_af3_price_forecasting_noability_other</t>
+  </si>
+  <si>
+    <t>mfs_af3_price_forecasting_noability_sm</t>
+  </si>
+  <si>
+    <t>Quelles sont les raisons principales expliquant pourquoi vous auriez des difficultés à donner une estimation précise des prix pratiqués par vos fournisseurs le mois prochain ?</t>
+  </si>
+  <si>
+    <t>mfs_in3_accepted_payment_modality_other</t>
+  </si>
+  <si>
+    <t>mfs_in3_accepted_payment_modality_sm</t>
+  </si>
+  <si>
+    <t>Quels types de paiement avez-vous acceptés de la part de vos clients ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_risque_type_paiement_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_risque_type_paiement_sm</t>
+  </si>
+  <si>
+    <t>Quel est le risque associé aux types de paiement que vous avez sélectionnés ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_type_paiement_refusee_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_type_paiement_refusee_sm</t>
+  </si>
+  <si>
+    <t>Y a-t-il des types de paiement que vous n'avez pas pu ou pas voulu accepter de la part de vos clients ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_difficulte_type_paiement_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_difficulte_type_paiement_sm</t>
+  </si>
+  <si>
+    <t>Pourquoi ces types de paiement sont-ils difficiles à accepter pour vous ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_existence_service_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_existence_service_sm</t>
+  </si>
+  <si>
+    <t>Y a-t-il des services de transfet monétaire (banques, micro finance, mobile money) dans votre commune, et si oui lesquelles ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_argent_mobile_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_argent_mobile_so</t>
+  </si>
+  <si>
+    <t>Comment décririez-vous votre niveau actuel d'accès à l'argent mobile ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_psf_informel_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_psf_informel_sm</t>
+  </si>
+  <si>
+    <t>Au cours des 30 derniers jours, quels services ou moyens avez-vous utilisés pour accéder à des espèces ou effectuer des transferts d'argent ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_especes_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_acces_especes_so</t>
+  </si>
+  <si>
+    <t>Comment décririez-vous votre niveau actuel d'accès aux espèces ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_equite_distribution_cva_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_equite_distribution_cva_sm</t>
+  </si>
+  <si>
+    <t>À votre avis, les habitants de cette commune estiment-ils que les transferts monétaires (CVA) sont distribués de manière juste et équitable ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_preference_coupon_cva_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_preference_coupon_cva_so</t>
+  </si>
+  <si>
+    <t>Si vous deviez travailler avec un fournisseur d'aide financière humanitaire (CVA), quel serait votre type de coupon préféré ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_risque_cva_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_risque_cva_sm</t>
+  </si>
+  <si>
+    <t>À votre avis, existe-t-il des risques associés aux transferts monétaires ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_tensions_sociales_cva_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_tensions_sociales_cva_sm</t>
+  </si>
+  <si>
+    <t>Si « Tensions sociales », quelles sont les tensions sociales qui découlent des transferts monétaires ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_impact_cva_autre_tx</t>
+  </si>
+  <si>
+    <t>CAR_cfa_impact_cva_sm</t>
+  </si>
+  <si>
+    <t>Quel serait l'impact de la fourniture d'une aide monétaire humanitaire aux ménages de cette commune sur votre commerce et sur le marché local ?</t>
+  </si>
+  <si>
+    <t>CAR_cfa_info_supplementaire_tx</t>
+  </si>
+  <si>
+    <t>Avez-vous des informations supplémentaires que vous souhaiteriez partager concernant le marché et votre perception de l'aide financière humanitaire (CVA) qui n'auraient pas été abordées dans cette enquête ?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -382,6 +389,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -663,11 +679,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="37.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -678,7 +697,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -689,7 +708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -700,7 +719,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -711,7 +730,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -722,7 +741,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -733,7 +752,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -744,7 +763,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -755,7 +774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -766,7 +785,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -777,7 +796,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -788,7 +807,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -799,7 +818,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -810,7 +829,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -821,7 +840,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -832,7 +851,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -843,7 +862,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -854,7 +873,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -865,7 +884,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -876,7 +895,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -887,7 +906,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -898,7 +917,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -909,7 +928,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -920,7 +939,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -931,7 +950,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -942,7 +961,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -953,7 +972,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>65</v>
       </c>
@@ -964,7 +983,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -975,7 +994,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>71</v>
       </c>
@@ -986,7 +1005,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>74</v>
       </c>
@@ -997,7 +1016,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>77</v>
       </c>
@@ -1008,7 +1027,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -1019,7 +1038,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>83</v>
       </c>
@@ -1030,7 +1049,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>86</v>
       </c>
@@ -1041,7 +1060,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>89</v>
       </c>
@@ -1052,7 +1071,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>92</v>
       </c>
@@ -1063,7 +1082,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>95</v>
       </c>
@@ -1074,7 +1093,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -1085,7 +1104,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>101</v>
       </c>
@@ -1096,7 +1115,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>104</v>
       </c>
@@ -1107,7 +1126,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>107</v>
       </c>
@@ -1120,6 +1139,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>